<commit_message>
preliminary completion of biomass integration in EnergyProduction
</commit_message>
<xml_diff>
--- a/sisepuede/ref/data_tables_and_derivations/ENERGY/energy_inputs_to_model_with_fuel_conversion_factors.xlsx
+++ b/sisepuede/ref/data_tables_and_derivations/ENERGY/energy_inputs_to_model_with_fuel_conversion_factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jsyme/Documents/Projects/git_jbus/sisepuede/ref/data_tables_and_derivations/ENERGY/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/usuario/git/sisepuede/sisepuede/ref/data_tables_and_derivations/ENERGY/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96776DEC-7A00-EB45-83B0-4B4613155A36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84DA2670-EDCC-FB4B-AE2E-96BE3FB44302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4320" yWindow="500" windowWidth="26300" windowHeight="20260" firstSheet="4" activeTab="10" xr2:uid="{5FFDFBED-0EDA-184B-B159-D6A0BE4DEBC4}"/>
+    <workbookView xWindow="4060" yWindow="760" windowWidth="26300" windowHeight="20180" firstSheet="10" activeTab="16" xr2:uid="{5FFDFBED-0EDA-184B-B159-D6A0BE4DEBC4}"/>
   </bookViews>
   <sheets>
     <sheet name="intro" sheetId="2" r:id="rId1"/>
@@ -26,15 +26,16 @@
     <sheet name="fuel_production" sheetId="13" r:id="rId11"/>
     <sheet name="water borne transport effic" sheetId="12" r:id="rId12"/>
     <sheet name="uranium_price" sheetId="8" r:id="rId13"/>
-    <sheet name="biomass_price" sheetId="9" r:id="rId14"/>
-    <sheet name="natural_gas_price" sheetId="7" r:id="rId15"/>
-    <sheet name="prices" sheetId="14" r:id="rId16"/>
-    <sheet name="rail_efficiencies" sheetId="15" r:id="rId17"/>
-    <sheet name="aviation_freight" sheetId="17" r:id="rId18"/>
-    <sheet name="public_efficiencies" sheetId="16" r:id="rId19"/>
+    <sheet name="waste_fuel_price" sheetId="21" r:id="rId14"/>
+    <sheet name="biomass_price" sheetId="9" r:id="rId15"/>
+    <sheet name="natural_gas_price" sheetId="7" r:id="rId16"/>
+    <sheet name="prices" sheetId="14" r:id="rId17"/>
+    <sheet name="rail_efficiencies" sheetId="15" r:id="rId18"/>
+    <sheet name="aviation_freight" sheetId="17" r:id="rId19"/>
+    <sheet name="public_efficiencies" sheetId="16" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">prices!$A$1:$T$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">prices!$A$1:$T$26</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -79,7 +80,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="973" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="658">
   <si>
     <t>IEA World Energy Balance includes production by PJ. These sheets contain information to convert PJ to tonnes and m3 to tonnes</t>
   </si>
@@ -2197,6 +2198,20 @@
   </si>
   <si>
     <t>189MJ/kg hydrogen</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>https://www.factmr.com/report/1461/refuse-derived-fuel-market
+https://link.springer.com/article/10.1007/s10311-025-01889-6 (some ged numbers to consider)</t>
+  </si>
+  <si>
+    <t>Use $92.5/tonne (mean of 55-130) with GED of 10 gj/tonne =&gt; 9.25/gj
+use 0.947813395 mmbtu/gj -&gt; 9.25/947813395 = 9.75930499</t>
+  </si>
+  <si>
+    <t>USD/mmbtu</t>
   </si>
 </sst>
 </file>
@@ -2670,13 +2685,40 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2684,10 +2726,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2696,35 +2741,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2741,25 +2765,10 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2767,6 +2776,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -2947,6 +2962,55 @@
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>444500</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>762000</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>1101557</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{01776C6D-E5BC-4A52-3C49-35C681D308D8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13754100" y="9347200"/>
+          <a:ext cx="7772400" cy="1647657"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -3348,21 +3412,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="73"/>
-      <c r="J1" s="73"/>
-      <c r="K1" s="73"/>
-      <c r="L1" s="73"/>
-      <c r="M1" s="73"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
+      <c r="J1" s="61"/>
+      <c r="K1" s="61"/>
+      <c r="L1" s="61"/>
+      <c r="M1" s="61"/>
     </row>
     <row r="2" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
@@ -3463,7 +3527,7 @@
       <c r="D10" s="33"/>
       <c r="E10" s="33"/>
       <c r="F10" s="33"/>
-      <c r="G10" s="79" t="s">
+      <c r="G10" s="82" t="s">
         <v>185</v>
       </c>
       <c r="J10" t="s">
@@ -3483,7 +3547,7 @@
       <c r="D11" s="33"/>
       <c r="E11" s="33"/>
       <c r="F11" s="33"/>
-      <c r="G11" s="79"/>
+      <c r="G11" s="82"/>
     </row>
     <row r="12" spans="1:13" ht="17" x14ac:dyDescent="0.2">
       <c r="A12" s="28">
@@ -3501,7 +3565,7 @@
       <c r="D12" s="33"/>
       <c r="E12" s="33"/>
       <c r="F12" s="33"/>
-      <c r="G12" s="79"/>
+      <c r="G12" s="82"/>
       <c r="J12">
         <v>0.09</v>
       </c>
@@ -3534,7 +3598,7 @@
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
-      <c r="G13" s="79"/>
+      <c r="G13" s="82"/>
       <c r="J13">
         <f>8.07/0.09</f>
         <v>89.666666666666671</v>
@@ -3560,7 +3624,7 @@
       </c>
       <c r="E14" s="33"/>
       <c r="F14" s="33"/>
-      <c r="G14" s="79"/>
+      <c r="G14" s="82"/>
       <c r="J14">
         <f>1060/J13</f>
         <v>11.821561338289962</v>
@@ -3628,19 +3692,19 @@
       </c>
     </row>
     <row r="41" spans="1:11" ht="21" x14ac:dyDescent="0.2">
-      <c r="A41" s="73" t="s">
+      <c r="A41" s="61" t="s">
         <v>314</v>
       </c>
-      <c r="B41" s="73"/>
-      <c r="C41" s="73"/>
-      <c r="D41" s="73"/>
-      <c r="E41" s="73"/>
-      <c r="F41" s="73"/>
-      <c r="G41" s="73"/>
-      <c r="H41" s="73"/>
-      <c r="I41" s="73"/>
-      <c r="J41" s="73"/>
-      <c r="K41" s="73"/>
+      <c r="B41" s="61"/>
+      <c r="C41" s="61"/>
+      <c r="D41" s="61"/>
+      <c r="E41" s="61"/>
+      <c r="F41" s="61"/>
+      <c r="G41" s="61"/>
+      <c r="H41" s="61"/>
+      <c r="I41" s="61"/>
+      <c r="J41" s="61"/>
+      <c r="K41" s="61"/>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
@@ -3675,7 +3739,7 @@
         <f>1/8.07</f>
         <v>0.12391573729863692</v>
       </c>
-      <c r="G47" s="72" t="s">
+      <c r="G47" s="65" t="s">
         <v>289</v>
       </c>
     </row>
@@ -3694,7 +3758,7 @@
         <f>1.06*E47</f>
         <v>0.13135068153655513</v>
       </c>
-      <c r="G48" s="72"/>
+      <c r="G48" s="65"/>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
@@ -3711,7 +3775,7 @@
         <f>E48*1.1</f>
         <v>0.14448574969021066</v>
       </c>
-      <c r="G49" s="72"/>
+      <c r="G49" s="65"/>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
@@ -3727,7 +3791,7 @@
       <c r="E50">
         <v>6</v>
       </c>
-      <c r="G50" s="72"/>
+      <c r="G50" s="65"/>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
@@ -3758,16 +3822,16 @@
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="D54" s="39"/>
-      <c r="E54" s="80" t="s">
+      <c r="E54" s="83" t="s">
         <v>290</v>
       </c>
-      <c r="F54" s="80"/>
-      <c r="G54" s="80"/>
-      <c r="H54" s="81" t="s">
+      <c r="F54" s="83"/>
+      <c r="G54" s="83"/>
+      <c r="H54" s="84" t="s">
         <v>294</v>
       </c>
-      <c r="I54" s="81"/>
-      <c r="J54" s="81"/>
+      <c r="I54" s="84"/>
+      <c r="J54" s="84"/>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
@@ -3945,29 +4009,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="67" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="84" t="s">
+      <c r="A1" s="60" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="K1" s="82" t="s">
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+      <c r="H1" s="60"/>
+      <c r="I1" s="60"/>
+      <c r="K1" s="58" t="s">
         <v>222</v>
       </c>
       <c r="L1" s="27" t="s">
         <v>156</v>
       </c>
-      <c r="S1" s="82" t="s">
+      <c r="S1" s="58" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="K2" s="82"/>
+      <c r="K2" s="58"/>
       <c r="M2" t="s">
         <v>225</v>
       </c>
@@ -3977,21 +4041,21 @@
       <c r="O2" t="s">
         <v>227</v>
       </c>
-      <c r="S2" s="82"/>
+      <c r="S2" s="58"/>
     </row>
     <row r="3" spans="1:21" ht="21" x14ac:dyDescent="0.25">
-      <c r="A3" s="83" t="s">
+      <c r="A3" s="59" t="s">
         <v>220</v>
       </c>
-      <c r="B3" s="83"/>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-      <c r="F3" s="83"/>
-      <c r="G3" s="83"/>
-      <c r="H3" s="83"/>
-      <c r="I3" s="83"/>
-      <c r="K3" s="82"/>
+      <c r="B3" s="59"/>
+      <c r="C3" s="59"/>
+      <c r="D3" s="59"/>
+      <c r="E3" s="59"/>
+      <c r="F3" s="59"/>
+      <c r="G3" s="59"/>
+      <c r="H3" s="59"/>
+      <c r="I3" s="59"/>
+      <c r="K3" s="58"/>
       <c r="L3" t="s">
         <v>159</v>
       </c>
@@ -4004,7 +4068,7 @@
       <c r="O3">
         <v>0</v>
       </c>
-      <c r="S3" s="82"/>
+      <c r="S3" s="58"/>
       <c r="T3" t="s">
         <v>159</v>
       </c>
@@ -4029,7 +4093,7 @@
       <c r="E4" s="27" t="s">
         <v>149</v>
       </c>
-      <c r="K4" s="82"/>
+      <c r="K4" s="58"/>
       <c r="L4" t="s">
         <v>158</v>
       </c>
@@ -4044,7 +4108,7 @@
         <f>N4/SUM(N$4:N$6)</f>
         <v>0.5</v>
       </c>
-      <c r="S4" s="82"/>
+      <c r="S4" s="58"/>
       <c r="T4" t="s">
         <v>158</v>
       </c>
@@ -4061,7 +4125,7 @@
         <v>1.0050251256281406</v>
       </c>
       <c r="C5">
-        <f t="shared" ref="B5:C5" si="0">1/(1-C4)</f>
+        <f t="shared" ref="C5" si="0">1/(1-C4)</f>
         <v>1.0416666666666667</v>
       </c>
       <c r="D5">
@@ -4071,7 +4135,7 @@
       <c r="I5" t="s">
         <v>237</v>
       </c>
-      <c r="K5" s="82"/>
+      <c r="K5" s="58"/>
       <c r="L5" t="s">
         <v>160</v>
       </c>
@@ -4086,7 +4150,7 @@
         <f>N5/SUM(N$4:N$6)</f>
         <v>0.47058823529411764</v>
       </c>
-      <c r="S5" s="82"/>
+      <c r="S5" s="58"/>
       <c r="T5" t="s">
         <v>160</v>
       </c>
@@ -4117,7 +4181,7 @@
         <f>E6*D6</f>
         <v>1.0043063938618926</v>
       </c>
-      <c r="K6" s="82"/>
+      <c r="K6" s="58"/>
       <c r="L6" t="s">
         <v>161</v>
       </c>
@@ -4132,7 +4196,7 @@
         <f t="shared" si="1"/>
         <v>2.9411764705882353E-2</v>
       </c>
-      <c r="S6" s="82"/>
+      <c r="S6" s="58"/>
       <c r="T6" t="s">
         <v>161</v>
       </c>
@@ -4268,17 +4332,17 @@
       </c>
     </row>
     <row r="13" spans="1:21" ht="21" x14ac:dyDescent="0.25">
-      <c r="A13" s="83" t="s">
+      <c r="A13" s="59" t="s">
         <v>232</v>
       </c>
-      <c r="B13" s="83"/>
-      <c r="C13" s="83"/>
-      <c r="D13" s="83"/>
-      <c r="E13" s="83"/>
-      <c r="F13" s="83"/>
-      <c r="G13" s="83"/>
-      <c r="H13" s="83"/>
-      <c r="I13" s="83"/>
+      <c r="B13" s="59"/>
+      <c r="C13" s="59"/>
+      <c r="D13" s="59"/>
+      <c r="E13" s="59"/>
+      <c r="F13" s="59"/>
+      <c r="G13" s="59"/>
+      <c r="H13" s="59"/>
+      <c r="I13" s="59"/>
       <c r="T13" t="s">
         <v>161</v>
       </c>
@@ -4424,17 +4488,17 @@
       </c>
     </row>
     <row r="23" spans="1:24" ht="21" x14ac:dyDescent="0.25">
-      <c r="A23" s="83" t="s">
+      <c r="A23" s="59" t="s">
         <v>231</v>
       </c>
-      <c r="B23" s="83"/>
-      <c r="C23" s="83"/>
-      <c r="D23" s="83"/>
-      <c r="E23" s="83"/>
-      <c r="F23" s="83"/>
-      <c r="G23" s="83"/>
-      <c r="H23" s="83"/>
-      <c r="I23" s="83"/>
+      <c r="B23" s="59"/>
+      <c r="C23" s="59"/>
+      <c r="D23" s="59"/>
+      <c r="E23" s="59"/>
+      <c r="F23" s="59"/>
+      <c r="G23" s="59"/>
+      <c r="H23" s="59"/>
+      <c r="I23" s="59"/>
       <c r="O23" s="23" t="s">
         <v>239</v>
       </c>
@@ -4810,17 +4874,17 @@
       </c>
     </row>
     <row r="33" spans="1:24" ht="21" x14ac:dyDescent="0.25">
-      <c r="A33" s="83" t="s">
+      <c r="A33" s="59" t="s">
         <v>229</v>
       </c>
-      <c r="B33" s="83"/>
-      <c r="C33" s="83"/>
-      <c r="D33" s="83"/>
-      <c r="E33" s="83"/>
-      <c r="F33" s="83"/>
-      <c r="G33" s="83"/>
-      <c r="H33" s="83"/>
-      <c r="I33" s="83"/>
+      <c r="B33" s="59"/>
+      <c r="C33" s="59"/>
+      <c r="D33" s="59"/>
+      <c r="E33" s="59"/>
+      <c r="F33" s="59"/>
+      <c r="G33" s="59"/>
+      <c r="H33" s="59"/>
+      <c r="I33" s="59"/>
       <c r="O33" s="23" t="s">
         <v>239</v>
       </c>
@@ -5320,17 +5384,17 @@
       </c>
     </row>
     <row r="54" spans="1:24" ht="31" x14ac:dyDescent="0.2">
-      <c r="A54" s="84" t="s">
+      <c r="A54" s="60" t="s">
         <v>281</v>
       </c>
-      <c r="B54" s="84"/>
-      <c r="C54" s="84"/>
-      <c r="D54" s="84"/>
-      <c r="E54" s="84"/>
-      <c r="F54" s="84"/>
-      <c r="G54" s="84"/>
-      <c r="H54" s="84"/>
-      <c r="I54" s="84"/>
+      <c r="B54" s="60"/>
+      <c r="C54" s="60"/>
+      <c r="D54" s="60"/>
+      <c r="E54" s="60"/>
+      <c r="F54" s="60"/>
+      <c r="G54" s="60"/>
+      <c r="H54" s="60"/>
+      <c r="I54" s="60"/>
       <c r="O54" s="23" t="s">
         <v>239</v>
       </c>
@@ -5367,17 +5431,17 @@
       </c>
     </row>
     <row r="56" spans="1:24" ht="21" x14ac:dyDescent="0.25">
-      <c r="A56" s="83" t="s">
+      <c r="A56" s="59" t="s">
         <v>282</v>
       </c>
-      <c r="B56" s="83"/>
-      <c r="C56" s="83"/>
-      <c r="D56" s="83"/>
-      <c r="E56" s="83"/>
-      <c r="F56" s="83"/>
-      <c r="G56" s="83"/>
-      <c r="H56" s="83"/>
-      <c r="I56" s="83"/>
+      <c r="B56" s="59"/>
+      <c r="C56" s="59"/>
+      <c r="D56" s="59"/>
+      <c r="E56" s="59"/>
+      <c r="F56" s="59"/>
+      <c r="G56" s="59"/>
+      <c r="H56" s="59"/>
+      <c r="I56" s="59"/>
       <c r="O56" s="23" t="s">
         <v>239</v>
       </c>
@@ -5504,7 +5568,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="66" t="s">
         <v>190</v>
       </c>
       <c r="B1" t="s">
@@ -5534,7 +5598,7 @@
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="64"/>
+      <c r="A2" s="66"/>
       <c r="B2" t="s">
         <v>189</v>
       </c>
@@ -5555,7 +5619,7 @@
       <c r="S2" s="36"/>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A3" s="64"/>
+      <c r="A3" s="66"/>
       <c r="B3" t="s">
         <v>162</v>
       </c>
@@ -6010,14 +6074,14 @@
       <c r="S29" s="36"/>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="G30" s="72" t="s">
+      <c r="G30" s="65" t="s">
         <v>192</v>
       </c>
-      <c r="H30" s="72"/>
-      <c r="I30" s="72"/>
-      <c r="J30" s="72"/>
-      <c r="K30" s="72"/>
-      <c r="L30" s="72"/>
+      <c r="H30" s="65"/>
+      <c r="I30" s="65"/>
+      <c r="J30" s="65"/>
+      <c r="K30" s="65"/>
+      <c r="L30" s="65"/>
       <c r="N30" s="36"/>
       <c r="O30" s="36"/>
       <c r="P30" s="36"/>
@@ -6050,14 +6114,14 @@
       <c r="S33" s="36"/>
     </row>
     <row r="34" spans="14:19" x14ac:dyDescent="0.2">
-      <c r="N34" s="72" t="s">
+      <c r="N34" s="65" t="s">
         <v>191</v>
       </c>
-      <c r="O34" s="72"/>
-      <c r="P34" s="72"/>
-      <c r="Q34" s="72"/>
-      <c r="R34" s="72"/>
-      <c r="S34" s="72"/>
+      <c r="O34" s="65"/>
+      <c r="P34" s="65"/>
+      <c r="Q34" s="65"/>
+      <c r="R34" s="65"/>
+      <c r="S34" s="65"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -6125,6 +6189,21 @@
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32020820-F468-184D-B040-2CFAE3A08EF1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>654</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D120EC9-D6D3-9A41-9D33-D74B19414CA1}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6166,7 +6245,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55C57F77-52F2-1B41-A795-B311D051266D}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -6184,14 +6263,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BF55BFE-4088-1E41-9DDD-2CBCBD9293D5}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:X26"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="7" max="11" width="0" hidden="1" customWidth="1"/>
     <col min="21" max="21" width="12.1640625" customWidth="1"/>
+    <col min="22" max="22" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
@@ -6262,7 +6341,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="2" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>357</v>
       </c>
@@ -6312,7 +6391,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="3" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>365</v>
       </c>
@@ -6396,7 +6475,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="5" spans="1:24" ht="23" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:24" ht="23" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>376</v>
       </c>
@@ -6489,7 +6568,7 @@
         <v>463</v>
       </c>
     </row>
-    <row r="7" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>386</v>
       </c>
@@ -6540,7 +6619,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="8" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>393</v>
       </c>
@@ -6594,7 +6673,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="9" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>398</v>
       </c>
@@ -6648,7 +6727,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="10" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>402</v>
       </c>
@@ -6677,7 +6756,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>405</v>
       </c>
@@ -6731,7 +6810,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="12" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>408</v>
       </c>
@@ -6885,7 +6964,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="15" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>422</v>
       </c>
@@ -6914,7 +6993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:24" hidden="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>425</v>
       </c>
@@ -6968,7 +7047,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="17" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>428</v>
       </c>
@@ -7022,7 +7101,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="18" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>433</v>
       </c>
@@ -7076,7 +7155,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="19" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>438</v>
       </c>
@@ -7105,7 +7184,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>441</v>
       </c>
@@ -7134,7 +7213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>444</v>
       </c>
@@ -7163,7 +7242,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>447</v>
       </c>
@@ -7192,7 +7271,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>450</v>
       </c>
@@ -7221,7 +7300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>453</v>
       </c>
@@ -7250,7 +7329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:20" ht="272" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>456</v>
       </c>
@@ -7278,8 +7357,20 @@
       <c r="L25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:20" hidden="1" x14ac:dyDescent="0.2">
+      <c r="M25">
+        <v>9.76</v>
+      </c>
+      <c r="N25" t="s">
+        <v>657</v>
+      </c>
+      <c r="Q25" s="5" t="s">
+        <v>655</v>
+      </c>
+      <c r="T25" s="5" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>459</v>
       </c>
@@ -7307,15 +7398,12 @@
       <c r="L26">
         <v>0</v>
       </c>
+      <c r="Q26">
+        <v>92.5</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T26" xr:uid="{5BF55BFE-4088-1E41-9DDD-2CBCBD9293D5}">
-    <filterColumn colId="15">
-      <filters>
-        <filter val="GRAVIMETRIC"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:T26" xr:uid="{5BF55BFE-4088-1E41-9DDD-2CBCBD9293D5}"/>
   <hyperlinks>
     <hyperlink ref="Q2" r:id="rId1" xr:uid="{97B41050-CC9F-4546-9AC9-366B7CD147F1}"/>
     <hyperlink ref="Q6" r:id="rId2" xr:uid="{08FFC797-A2CA-EB42-AD8A-C4509A958662}"/>
@@ -7324,10 +7412,11 @@
     <hyperlink ref="X13" r:id="rId5" xr:uid="{005914C0-4251-9446-BF49-FD4ECEEDB527}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId6"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8F50D75-3216-704D-87F9-6F7CF1AE4454}">
   <dimension ref="A1:K75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -7396,32 +7485,32 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="87" t="s">
+      <c r="A13" s="90" t="s">
         <v>504</v>
       </c>
-      <c r="B13" s="87"/>
-      <c r="C13" s="87"/>
-      <c r="D13" s="87"/>
-      <c r="E13" s="87"/>
-      <c r="F13" s="87"/>
-      <c r="G13" s="87"/>
-      <c r="H13" s="87"/>
-      <c r="I13" s="87"/>
-      <c r="J13" s="87"/>
+      <c r="B13" s="90"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="90"/>
+      <c r="E13" s="90"/>
+      <c r="F13" s="90"/>
+      <c r="G13" s="90"/>
+      <c r="H13" s="90"/>
+      <c r="I13" s="90"/>
+      <c r="J13" s="90"/>
     </row>
     <row r="17" spans="1:11" ht="26" x14ac:dyDescent="0.3">
-      <c r="A17" s="88" t="s">
+      <c r="A17" s="89" t="s">
         <v>504</v>
       </c>
-      <c r="B17" s="88"/>
-      <c r="C17" s="88"/>
-      <c r="D17" s="88"/>
-      <c r="E17" s="88"/>
-      <c r="F17" s="88"/>
-      <c r="G17" s="88"/>
-      <c r="H17" s="88"/>
-      <c r="I17" s="88"/>
-      <c r="J17" s="88"/>
+      <c r="B17" s="89"/>
+      <c r="C17" s="89"/>
+      <c r="D17" s="89"/>
+      <c r="E17" s="89"/>
+      <c r="F17" s="89"/>
+      <c r="G17" s="89"/>
+      <c r="H17" s="89"/>
+      <c r="I17" s="89"/>
+      <c r="J17" s="89"/>
     </row>
     <row r="18" spans="1:11" ht="26" x14ac:dyDescent="0.3">
       <c r="A18" s="47"/>
@@ -7436,25 +7525,25 @@
       <c r="J18" s="47"/>
     </row>
     <row r="19" spans="1:11" ht="104" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="89" t="s">
+      <c r="A19" s="87" t="s">
         <v>506</v>
       </c>
-      <c r="B19" s="90"/>
-      <c r="C19" s="90"/>
-      <c r="D19" s="90"/>
-      <c r="E19" s="90"/>
-      <c r="F19" s="90"/>
-      <c r="G19" s="90"/>
-      <c r="H19" s="90"/>
-      <c r="I19" s="90"/>
+      <c r="B19" s="88"/>
+      <c r="C19" s="88"/>
+      <c r="D19" s="88"/>
+      <c r="E19" s="88"/>
+      <c r="F19" s="88"/>
+      <c r="G19" s="88"/>
+      <c r="H19" s="88"/>
+      <c r="I19" s="88"/>
     </row>
     <row r="21" spans="1:11" ht="84" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="67" t="s">
+      <c r="A21" s="64" t="s">
         <v>495</v>
       </c>
-      <c r="B21" s="67"/>
-      <c r="C21" s="67"/>
-      <c r="D21" s="67"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="64"/>
+      <c r="D21" s="64"/>
       <c r="K21">
         <f>47951850/5462141</f>
         <v>8.7789476690550465</v>
@@ -7480,7 +7569,7 @@
       <c r="B25" t="s">
         <v>496</v>
       </c>
-      <c r="C25" s="80" t="s">
+      <c r="C25" s="83" t="s">
         <v>500</v>
       </c>
     </row>
@@ -7491,7 +7580,7 @@
       <c r="B26" t="s">
         <v>498</v>
       </c>
-      <c r="C26" s="80"/>
+      <c r="C26" s="83"/>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27">
@@ -7501,7 +7590,7 @@
       <c r="B27" t="s">
         <v>497</v>
       </c>
-      <c r="C27" s="80"/>
+      <c r="C27" s="83"/>
       <c r="G27">
         <f>1/8.8</f>
         <v>0.11363636363636363</v>
@@ -7515,7 +7604,7 @@
       <c r="B28" t="s">
         <v>489</v>
       </c>
-      <c r="C28" s="80"/>
+      <c r="C28" s="83"/>
       <c r="D28">
         <f>8.8/6806</f>
         <v>1.2929767851895388E-3</v>
@@ -7529,7 +7618,7 @@
       <c r="B29" t="s">
         <v>499</v>
       </c>
-      <c r="C29" s="80"/>
+      <c r="C29" s="83"/>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32">
@@ -7538,7 +7627,7 @@
       <c r="B32" t="s">
         <v>503</v>
       </c>
-      <c r="C32" s="80" t="s">
+      <c r="C32" s="83" t="s">
         <v>201</v>
       </c>
       <c r="D32" t="s">
@@ -7556,7 +7645,7 @@
       <c r="B33" t="s">
         <v>499</v>
       </c>
-      <c r="C33" s="80"/>
+      <c r="C33" s="83"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="18">
@@ -7566,7 +7655,7 @@
       <c r="B34" t="s">
         <v>488</v>
       </c>
-      <c r="C34" s="80"/>
+      <c r="C34" s="83"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="C36" t="s">
@@ -7574,17 +7663,17 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="104" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="89" t="s">
+      <c r="A39" s="87" t="s">
         <v>507</v>
       </c>
-      <c r="B39" s="90"/>
-      <c r="C39" s="90"/>
-      <c r="D39" s="90"/>
-      <c r="E39" s="90"/>
-      <c r="F39" s="90"/>
-      <c r="G39" s="90"/>
-      <c r="H39" s="90"/>
-      <c r="I39" s="90"/>
+      <c r="B39" s="88"/>
+      <c r="C39" s="88"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="88"/>
+      <c r="F39" s="88"/>
+      <c r="G39" s="88"/>
+      <c r="H39" s="88"/>
+      <c r="I39" s="88"/>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41">
@@ -7660,18 +7749,18 @@
       </c>
     </row>
     <row r="52" spans="1:10" ht="26" x14ac:dyDescent="0.3">
-      <c r="A52" s="88" t="s">
+      <c r="A52" s="89" t="s">
         <v>535</v>
       </c>
-      <c r="B52" s="88"/>
-      <c r="C52" s="88"/>
-      <c r="D52" s="88"/>
-      <c r="E52" s="88"/>
-      <c r="F52" s="88"/>
-      <c r="G52" s="88"/>
-      <c r="H52" s="88"/>
-      <c r="I52" s="88"/>
-      <c r="J52" s="88"/>
+      <c r="B52" s="89"/>
+      <c r="C52" s="89"/>
+      <c r="D52" s="89"/>
+      <c r="E52" s="89"/>
+      <c r="F52" s="89"/>
+      <c r="G52" s="89"/>
+      <c r="H52" s="89"/>
+      <c r="I52" s="89"/>
+      <c r="J52" s="89"/>
     </row>
     <row r="53" spans="1:10" ht="26" x14ac:dyDescent="0.3">
       <c r="A53" s="47"/>
@@ -7686,17 +7775,17 @@
       <c r="J53" s="47"/>
     </row>
     <row r="54" spans="1:10" ht="104" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="89" t="s">
+      <c r="A54" s="87" t="s">
         <v>507</v>
       </c>
-      <c r="B54" s="90"/>
-      <c r="C54" s="90"/>
-      <c r="D54" s="90"/>
-      <c r="E54" s="90"/>
-      <c r="F54" s="90"/>
-      <c r="G54" s="90"/>
-      <c r="H54" s="90"/>
-      <c r="I54" s="90"/>
+      <c r="B54" s="88"/>
+      <c r="C54" s="88"/>
+      <c r="D54" s="88"/>
+      <c r="E54" s="88"/>
+      <c r="F54" s="88"/>
+      <c r="G54" s="88"/>
+      <c r="H54" s="88"/>
+      <c r="I54" s="88"/>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57">
@@ -7706,7 +7795,7 @@
       <c r="B57" t="s">
         <v>508</v>
       </c>
-      <c r="C57" s="80" t="s">
+      <c r="C57" s="83" t="s">
         <v>201</v>
       </c>
     </row>
@@ -7718,7 +7807,7 @@
       <c r="B58" t="s">
         <v>488</v>
       </c>
-      <c r="C58" s="80"/>
+      <c r="C58" s="83"/>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60">
@@ -7845,22 +7934,22 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="C25:C29"/>
+    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="A17:J17"/>
+    <mergeCell ref="A19:I19"/>
     <mergeCell ref="A39:I39"/>
     <mergeCell ref="C32:C34"/>
     <mergeCell ref="A52:J52"/>
     <mergeCell ref="A54:I54"/>
     <mergeCell ref="C57:C58"/>
-    <mergeCell ref="A21:D21"/>
-    <mergeCell ref="C25:C29"/>
-    <mergeCell ref="A13:J13"/>
-    <mergeCell ref="A17:J17"/>
-    <mergeCell ref="A19:I19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68D1AFF-A559-F545-B121-69B0DF3FAC36}">
   <dimension ref="A1:K27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -8583,213 +8672,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{201F496F-0260-FD4C-850F-564E18865F2A}">
-  <dimension ref="A9:O32"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="2" max="2" width="17.33203125" customWidth="1"/>
-    <col min="13" max="15" width="25.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="9" spans="1:10" ht="26" x14ac:dyDescent="0.3">
-      <c r="A9" s="88" t="s">
-        <v>514</v>
-      </c>
-      <c r="B9" s="88"/>
-      <c r="C9" s="88"/>
-      <c r="D9" s="88"/>
-      <c r="E9" s="88"/>
-      <c r="F9" s="88"/>
-      <c r="G9" s="88"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="88"/>
-      <c r="J9" s="88"/>
-    </row>
-    <row r="10" spans="1:10" ht="26" x14ac:dyDescent="0.3">
-      <c r="A10" s="47"/>
-      <c r="B10" s="47"/>
-      <c r="C10" s="47"/>
-      <c r="D10" s="47"/>
-      <c r="E10" s="47"/>
-      <c r="F10" s="47"/>
-      <c r="G10" s="47"/>
-      <c r="H10" s="47"/>
-      <c r="I10" s="47"/>
-      <c r="J10" s="47"/>
-    </row>
-    <row r="11" spans="1:10" ht="104" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="89" t="s">
-        <v>515</v>
-      </c>
-      <c r="B11" s="90"/>
-      <c r="C11" s="90"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="90"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="90"/>
-      <c r="H11" s="90"/>
-      <c r="I11" s="90"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>518</v>
-      </c>
-      <c r="B14" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>0.19</v>
-      </c>
-      <c r="B17" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18">
-        <f>C32</f>
-        <v>71.146490917702906</v>
-      </c>
-      <c r="B18" t="s">
-        <v>534</v>
-      </c>
-      <c r="C18" t="s">
-        <v>522</v>
-      </c>
-      <c r="D18" t="s">
-        <v>523</v>
-      </c>
-      <c r="M18" s="76" t="s">
-        <v>521</v>
-      </c>
-      <c r="N18" s="76"/>
-      <c r="O18" s="76"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C19">
-        <v>25.8</v>
-      </c>
-      <c r="D19">
-        <v>0.5</v>
-      </c>
-      <c r="E19" t="s">
-        <v>524</v>
-      </c>
-      <c r="M19" s="76"/>
-      <c r="N19" s="76"/>
-      <c r="O19" s="76"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C20">
-        <v>59.7</v>
-      </c>
-      <c r="D20">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="E20" t="s">
-        <v>525</v>
-      </c>
-      <c r="M20" s="76"/>
-      <c r="N20" s="76"/>
-      <c r="O20" s="76"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C21">
-        <v>82</v>
-      </c>
-      <c r="D21">
-        <v>0.10199999999999999</v>
-      </c>
-      <c r="E21" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C23" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C24" t="s">
-        <v>528</v>
-      </c>
-      <c r="D24" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="25" spans="1:15" ht="17" x14ac:dyDescent="0.25">
-      <c r="C25" s="48">
-        <v>-7.0092399999999999E-3</v>
-      </c>
-      <c r="D25">
-        <v>0.68868282999999997</v>
-      </c>
-    </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C27" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C28">
-        <f>1/C25</f>
-        <v>-142.66882001472342</v>
-      </c>
-      <c r="D28">
-        <f>D25/C25</f>
-        <v>-98.253566720500359</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C30">
-        <f>D19*C28-D28</f>
-        <v>26.919156713138648</v>
-      </c>
-      <c r="D30" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="C31">
-        <f>D20*C28-D28</f>
-        <v>56.879608916230566</v>
-      </c>
-      <c r="D31" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B32" t="s">
-        <v>531</v>
-      </c>
-      <c r="C32">
-        <f>C28*A17-D28</f>
-        <v>71.146490917702906</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A9:J9"/>
-    <mergeCell ref="A11:I11"/>
-    <mergeCell ref="M18:O20"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{881E6503-80B4-134F-BEAF-440BF1CB0F2D}">
   <dimension ref="A1:V81"/>
@@ -8912,19 +8794,19 @@
       <c r="C10" s="1"/>
     </row>
     <row r="11" spans="1:22" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="73" t="s">
+      <c r="A11" s="61" t="s">
         <v>142</v>
       </c>
-      <c r="B11" s="73"/>
-      <c r="C11" s="73"/>
-      <c r="D11" s="73"/>
-      <c r="E11" s="73"/>
-      <c r="F11" s="73"/>
-      <c r="G11" s="73"/>
-      <c r="H11" s="73"/>
-      <c r="I11" s="73"/>
-      <c r="J11" s="73"/>
-      <c r="K11" s="73"/>
+      <c r="B11" s="61"/>
+      <c r="C11" s="61"/>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="61"/>
+      <c r="G11" s="61"/>
+      <c r="H11" s="61"/>
+      <c r="I11" s="61"/>
+      <c r="J11" s="61"/>
+      <c r="K11" s="61"/>
       <c r="L11" t="s">
         <v>90</v>
       </c>
@@ -8948,42 +8830,42 @@
       </c>
     </row>
     <row r="15" spans="1:22" ht="174" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="76" t="s">
+      <c r="B15" s="63" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="76"/>
-      <c r="D15" s="76"/>
-      <c r="E15" s="76"/>
-      <c r="F15" s="76"/>
-      <c r="N15" s="67"/>
-      <c r="O15" s="67"/>
-      <c r="P15" s="67"/>
-      <c r="Q15" s="67"/>
-      <c r="R15" s="67"/>
-      <c r="S15" s="67"/>
-      <c r="T15" s="67"/>
-      <c r="U15" s="67"/>
-      <c r="V15" s="67"/>
+      <c r="C15" s="63"/>
+      <c r="D15" s="63"/>
+      <c r="E15" s="63"/>
+      <c r="F15" s="63"/>
+      <c r="N15" s="64"/>
+      <c r="O15" s="64"/>
+      <c r="P15" s="64"/>
+      <c r="Q15" s="64"/>
+      <c r="R15" s="64"/>
+      <c r="S15" s="64"/>
+      <c r="T15" s="64"/>
+      <c r="U15" s="64"/>
+      <c r="V15" s="64"/>
     </row>
     <row r="16" spans="1:22" ht="56" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="67" t="s">
+      <c r="B16" s="64" t="s">
         <v>84</v>
       </c>
-      <c r="C16" s="67"/>
-      <c r="D16" s="67"/>
-      <c r="E16" s="67"/>
-      <c r="F16" s="67"/>
-      <c r="I16" s="72"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="72"/>
-      <c r="L16" s="72"/>
+      <c r="C16" s="64"/>
+      <c r="D16" s="64"/>
+      <c r="E16" s="64"/>
+      <c r="F16" s="64"/>
+      <c r="I16" s="65"/>
+      <c r="J16" s="65"/>
+      <c r="K16" s="65"/>
+      <c r="L16" s="65"/>
       <c r="M16" s="6"/>
-      <c r="N16" s="68"/>
-      <c r="O16" s="68"/>
-      <c r="P16" s="68"/>
-      <c r="Q16" s="68"/>
-      <c r="R16" s="68"/>
-      <c r="S16" s="68"/>
+      <c r="N16" s="69"/>
+      <c r="O16" s="69"/>
+      <c r="P16" s="69"/>
+      <c r="Q16" s="69"/>
+      <c r="R16" s="69"/>
+      <c r="S16" s="69"/>
       <c r="T16" s="18"/>
       <c r="U16" s="18"/>
     </row>
@@ -9030,7 +8912,7 @@
       </c>
     </row>
     <row r="18" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A18" s="64" t="s">
+      <c r="A18" s="66" t="s">
         <v>88</v>
       </c>
       <c r="B18" t="s">
@@ -9084,7 +8966,7 @@
       </c>
     </row>
     <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="64"/>
+      <c r="A19" s="66"/>
       <c r="B19" t="s">
         <v>36</v>
       </c>
@@ -9136,7 +9018,7 @@
       </c>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A20" s="64"/>
+      <c r="A20" s="66"/>
       <c r="B20" t="s">
         <v>37</v>
       </c>
@@ -9188,7 +9070,7 @@
       </c>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A21" s="64"/>
+      <c r="A21" s="66"/>
       <c r="B21" s="8" t="s">
         <v>85</v>
       </c>
@@ -9237,7 +9119,7 @@
       <c r="S21" s="8"/>
     </row>
     <row r="22" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A22" s="64"/>
+      <c r="A22" s="66"/>
       <c r="B22" s="8" t="s">
         <v>86</v>
       </c>
@@ -9268,7 +9150,7 @@
       <c r="S22" s="8"/>
     </row>
     <row r="23" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A23" s="64"/>
+      <c r="A23" s="66"/>
       <c r="B23" s="8" t="s">
         <v>87</v>
       </c>
@@ -9300,7 +9182,7 @@
       <c r="S23" s="8"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A24" s="64"/>
+      <c r="A24" s="66"/>
       <c r="B24" t="s">
         <v>39</v>
       </c>
@@ -9324,7 +9206,7 @@
       <c r="A25" s="20"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="64" t="s">
+      <c r="A26" s="66" t="s">
         <v>89</v>
       </c>
       <c r="B26" t="s">
@@ -9347,7 +9229,7 @@
       </c>
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="64"/>
+      <c r="A27" s="66"/>
       <c r="B27" t="s">
         <v>91</v>
       </c>
@@ -9374,10 +9256,10 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C28" s="8"/>
-      <c r="N28" s="72"/>
-      <c r="O28" s="72"/>
-      <c r="P28" s="72"/>
-      <c r="Q28" s="72"/>
+      <c r="N28" s="65"/>
+      <c r="O28" s="65"/>
+      <c r="P28" s="65"/>
+      <c r="Q28" s="65"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.2">
       <c r="C29" s="8"/>
@@ -9395,14 +9277,14 @@
       </c>
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="J30" s="74" t="s">
+      <c r="J30" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="K30" s="61" t="s">
+      <c r="K30" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="L30" s="62"/>
-      <c r="M30" s="69"/>
+      <c r="L30" s="71"/>
+      <c r="M30" s="72"/>
       <c r="N30" s="9">
         <v>7.0000000000000007E-2</v>
       </c>
@@ -9417,12 +9299,12 @@
       </c>
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="J31" s="74"/>
-      <c r="K31" s="63" t="s">
+      <c r="J31" s="68"/>
+      <c r="K31" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="L31" s="64"/>
-      <c r="M31" s="70"/>
+      <c r="L31" s="66"/>
+      <c r="M31" s="74"/>
       <c r="N31" s="12">
         <v>0.83</v>
       </c>
@@ -9441,12 +9323,12 @@
         <f>(0.0022*0.037)^0.5</f>
         <v>9.0221948549119683E-3</v>
       </c>
-      <c r="J32" s="74"/>
-      <c r="K32" s="65" t="s">
+      <c r="J32" s="68"/>
+      <c r="K32" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="L32" s="66"/>
-      <c r="M32" s="71"/>
+      <c r="L32" s="76"/>
+      <c r="M32" s="77"/>
       <c r="N32" s="14">
         <v>0.1</v>
       </c>
@@ -9461,14 +9343,14 @@
       </c>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J33" s="60" t="s">
+      <c r="J33" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="K33" s="61" t="s">
+      <c r="K33" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="L33" s="62"/>
-      <c r="M33" s="69"/>
+      <c r="L33" s="71"/>
+      <c r="M33" s="72"/>
       <c r="N33" s="9">
         <v>0.09</v>
       </c>
@@ -9483,12 +9365,12 @@
       </c>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J34" s="60"/>
-      <c r="K34" s="63" t="s">
+      <c r="J34" s="67"/>
+      <c r="K34" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="L34" s="64"/>
-      <c r="M34" s="70"/>
+      <c r="L34" s="66"/>
+      <c r="M34" s="74"/>
       <c r="N34" s="12">
         <v>0.78</v>
       </c>
@@ -9503,12 +9385,12 @@
       </c>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J35" s="60"/>
-      <c r="K35" s="65" t="s">
+      <c r="J35" s="67"/>
+      <c r="K35" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="L35" s="66"/>
-      <c r="M35" s="71"/>
+      <c r="L35" s="76"/>
+      <c r="M35" s="77"/>
       <c r="N35" s="14">
         <v>0.13</v>
       </c>
@@ -9523,14 +9405,14 @@
       </c>
     </row>
     <row r="36" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J36" s="60" t="s">
+      <c r="J36" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="K36" s="61" t="s">
+      <c r="K36" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="L36" s="62"/>
-      <c r="M36" s="69"/>
+      <c r="L36" s="71"/>
+      <c r="M36" s="72"/>
       <c r="N36" s="9">
         <v>0.2</v>
       </c>
@@ -9545,12 +9427,12 @@
       </c>
     </row>
     <row r="37" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J37" s="60"/>
-      <c r="K37" s="63" t="s">
+      <c r="J37" s="67"/>
+      <c r="K37" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="L37" s="64"/>
-      <c r="M37" s="70"/>
+      <c r="L37" s="66"/>
+      <c r="M37" s="74"/>
       <c r="N37" s="12">
         <v>0.8</v>
       </c>
@@ -9565,12 +9447,12 @@
       </c>
     </row>
     <row r="38" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J38" s="60"/>
-      <c r="K38" s="65" t="s">
+      <c r="J38" s="67"/>
+      <c r="K38" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="L38" s="66"/>
-      <c r="M38" s="71"/>
+      <c r="L38" s="76"/>
+      <c r="M38" s="77"/>
       <c r="N38" s="12">
         <v>0</v>
       </c>
@@ -9585,14 +9467,14 @@
       </c>
     </row>
     <row r="39" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J39" s="60" t="s">
+      <c r="J39" s="67" t="s">
         <v>62</v>
       </c>
-      <c r="K39" s="61" t="s">
+      <c r="K39" s="70" t="s">
         <v>59</v>
       </c>
-      <c r="L39" s="62"/>
-      <c r="M39" s="62"/>
+      <c r="L39" s="71"/>
+      <c r="M39" s="71"/>
       <c r="N39" s="9">
         <f>AVERAGE(N30,N33,N36)</f>
         <v>0.12</v>
@@ -9611,12 +9493,12 @@
       </c>
     </row>
     <row r="40" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J40" s="60"/>
-      <c r="K40" s="63" t="s">
+      <c r="J40" s="67"/>
+      <c r="K40" s="73" t="s">
         <v>60</v>
       </c>
-      <c r="L40" s="64"/>
-      <c r="M40" s="64"/>
+      <c r="L40" s="66"/>
+      <c r="M40" s="66"/>
       <c r="N40" s="12">
         <f t="shared" ref="N40:Q41" si="5">AVERAGE(N31,N34,N37)</f>
         <v>0.80333333333333334</v>
@@ -9635,12 +9517,12 @@
       </c>
     </row>
     <row r="41" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="J41" s="60"/>
-      <c r="K41" s="65" t="s">
+      <c r="J41" s="67"/>
+      <c r="K41" s="75" t="s">
         <v>61</v>
       </c>
-      <c r="L41" s="66"/>
-      <c r="M41" s="66"/>
+      <c r="L41" s="76"/>
+      <c r="M41" s="76"/>
       <c r="N41" s="14">
         <f t="shared" si="5"/>
         <v>7.6666666666666675E-2</v>
@@ -9687,14 +9569,14 @@
       <c r="G43" t="s">
         <v>47</v>
       </c>
-      <c r="I43" s="59" t="s">
+      <c r="I43" s="79" t="s">
         <v>97</v>
       </c>
-      <c r="J43" s="59"/>
-      <c r="K43" s="59"/>
-      <c r="L43" s="59"/>
-      <c r="M43" s="59"/>
-      <c r="N43" s="58">
+      <c r="J43" s="79"/>
+      <c r="K43" s="79"/>
+      <c r="L43" s="79"/>
+      <c r="M43" s="79"/>
+      <c r="N43" s="78">
         <f>1-N42</f>
         <v>8.7121212121212155E-2</v>
       </c>
@@ -9719,12 +9601,12 @@
         <f>F43-F22-F23</f>
         <v>6.8000000000000027E-8</v>
       </c>
-      <c r="I44" s="59"/>
-      <c r="J44" s="59"/>
-      <c r="K44" s="59"/>
-      <c r="L44" s="59"/>
-      <c r="M44" s="59"/>
-      <c r="N44" s="58"/>
+      <c r="I44" s="79"/>
+      <c r="J44" s="79"/>
+      <c r="K44" s="79"/>
+      <c r="L44" s="79"/>
+      <c r="M44" s="79"/>
+      <c r="N44" s="78"/>
     </row>
     <row r="45" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
@@ -9841,19 +9723,19 @@
       </c>
     </row>
     <row r="51" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="73" t="s">
+      <c r="A51" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="B51" s="73"/>
-      <c r="C51" s="73"/>
-      <c r="D51" s="73"/>
-      <c r="E51" s="73"/>
-      <c r="F51" s="73"/>
-      <c r="G51" s="73"/>
-      <c r="H51" s="73"/>
-      <c r="I51" s="73"/>
-      <c r="J51" s="73"/>
-      <c r="K51" s="73"/>
+      <c r="B51" s="61"/>
+      <c r="C51" s="61"/>
+      <c r="D51" s="61"/>
+      <c r="E51" s="61"/>
+      <c r="F51" s="61"/>
+      <c r="G51" s="61"/>
+      <c r="H51" s="61"/>
+      <c r="I51" s="61"/>
+      <c r="J51" s="61"/>
+      <c r="K51" s="61"/>
     </row>
     <row r="52" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A52" s="26" t="s">
@@ -9872,19 +9754,19 @@
     </row>
     <row r="56" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="57" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="73" t="s">
+      <c r="A57" s="61" t="s">
         <v>144</v>
       </c>
-      <c r="B57" s="73"/>
-      <c r="C57" s="73"/>
-      <c r="D57" s="73"/>
-      <c r="E57" s="73"/>
-      <c r="F57" s="73"/>
-      <c r="G57" s="73"/>
-      <c r="H57" s="73"/>
-      <c r="I57" s="73"/>
-      <c r="J57" s="73"/>
-      <c r="K57" s="73"/>
+      <c r="B57" s="61"/>
+      <c r="C57" s="61"/>
+      <c r="D57" s="61"/>
+      <c r="E57" s="61"/>
+      <c r="F57" s="61"/>
+      <c r="G57" s="61"/>
+      <c r="H57" s="61"/>
+      <c r="I57" s="61"/>
+      <c r="J57" s="61"/>
+      <c r="K57" s="61"/>
     </row>
     <row r="58" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A58" s="26" t="s">
@@ -9910,34 +9792,34 @@
       </c>
     </row>
     <row r="64" spans="1:11" ht="21" x14ac:dyDescent="0.2">
-      <c r="A64" s="73" t="s">
+      <c r="A64" s="61" t="s">
         <v>280</v>
       </c>
-      <c r="B64" s="73"/>
-      <c r="C64" s="73"/>
-      <c r="D64" s="73"/>
-      <c r="E64" s="73"/>
-      <c r="F64" s="73"/>
-      <c r="G64" s="73"/>
-      <c r="H64" s="73"/>
-      <c r="I64" s="73"/>
-      <c r="J64" s="73"/>
-      <c r="K64" s="73"/>
+      <c r="B64" s="61"/>
+      <c r="C64" s="61"/>
+      <c r="D64" s="61"/>
+      <c r="E64" s="61"/>
+      <c r="F64" s="61"/>
+      <c r="G64" s="61"/>
+      <c r="H64" s="61"/>
+      <c r="I64" s="61"/>
+      <c r="J64" s="61"/>
+      <c r="K64" s="61"/>
     </row>
     <row r="71" spans="1:11" ht="21" x14ac:dyDescent="0.2">
-      <c r="A71" s="73" t="s">
+      <c r="A71" s="61" t="s">
         <v>315</v>
       </c>
-      <c r="B71" s="73"/>
-      <c r="C71" s="73"/>
-      <c r="D71" s="73"/>
-      <c r="E71" s="73"/>
-      <c r="F71" s="73"/>
-      <c r="G71" s="73"/>
-      <c r="H71" s="73"/>
-      <c r="I71" s="73"/>
-      <c r="J71" s="73"/>
-      <c r="K71" s="73"/>
+      <c r="B71" s="61"/>
+      <c r="C71" s="61"/>
+      <c r="D71" s="61"/>
+      <c r="E71" s="61"/>
+      <c r="F71" s="61"/>
+      <c r="G71" s="61"/>
+      <c r="H71" s="61"/>
+      <c r="I71" s="61"/>
+      <c r="J71" s="61"/>
+      <c r="K71" s="61"/>
     </row>
     <row r="72" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A72" s="26" t="s">
@@ -9950,10 +9832,10 @@
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A74" s="75" t="s">
+      <c r="A74" s="62" t="s">
         <v>309</v>
       </c>
-      <c r="B74" s="75"/>
+      <c r="B74" s="62"/>
       <c r="C74" s="42" t="s">
         <v>109</v>
       </c>
@@ -9978,10 +9860,10 @@
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A76" s="75" t="s">
+      <c r="A76" s="62" t="s">
         <v>317</v>
       </c>
-      <c r="B76" s="75"/>
+      <c r="B76" s="62"/>
       <c r="C76" s="41">
         <f>C75*$B$80</f>
         <v>2.6086956521739112E-4</v>
@@ -10052,21 +9934,12 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A71:K71"/>
-    <mergeCell ref="A74:B74"/>
-    <mergeCell ref="A76:B76"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="I16:L16"/>
-    <mergeCell ref="A64:K64"/>
-    <mergeCell ref="A57:K57"/>
-    <mergeCell ref="A11:K11"/>
-    <mergeCell ref="A51:K51"/>
-    <mergeCell ref="A18:A24"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="J36:J38"/>
-    <mergeCell ref="J33:J35"/>
-    <mergeCell ref="J30:J32"/>
+    <mergeCell ref="N43:N44"/>
+    <mergeCell ref="I43:M44"/>
+    <mergeCell ref="J39:J41"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="K40:M40"/>
+    <mergeCell ref="K41:M41"/>
     <mergeCell ref="N15:V15"/>
     <mergeCell ref="R16:S16"/>
     <mergeCell ref="K36:M36"/>
@@ -10080,12 +9953,21 @@
     <mergeCell ref="N28:Q28"/>
     <mergeCell ref="K34:M34"/>
     <mergeCell ref="K35:M35"/>
-    <mergeCell ref="N43:N44"/>
-    <mergeCell ref="I43:M44"/>
-    <mergeCell ref="J39:J41"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="K40:M40"/>
-    <mergeCell ref="K41:M41"/>
+    <mergeCell ref="A11:K11"/>
+    <mergeCell ref="A51:K51"/>
+    <mergeCell ref="A18:A24"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="J36:J38"/>
+    <mergeCell ref="J33:J35"/>
+    <mergeCell ref="J30:J32"/>
+    <mergeCell ref="A71:K71"/>
+    <mergeCell ref="A74:B74"/>
+    <mergeCell ref="A76:B76"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="I16:L16"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="A57:K57"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A55" r:id="rId1" xr:uid="{939BE22A-9CE0-E745-AEFB-468D46C49282}"/>
@@ -10094,6 +9976,213 @@
   <ignoredErrors>
     <ignoredError sqref="C22" formula="1"/>
   </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{201F496F-0260-FD4C-850F-564E18865F2A}">
+  <dimension ref="A9:O32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="13" max="15" width="25.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="9" spans="1:10" ht="26" x14ac:dyDescent="0.3">
+      <c r="A9" s="89" t="s">
+        <v>514</v>
+      </c>
+      <c r="B9" s="89"/>
+      <c r="C9" s="89"/>
+      <c r="D9" s="89"/>
+      <c r="E9" s="89"/>
+      <c r="F9" s="89"/>
+      <c r="G9" s="89"/>
+      <c r="H9" s="89"/>
+      <c r="I9" s="89"/>
+      <c r="J9" s="89"/>
+    </row>
+    <row r="10" spans="1:10" ht="26" x14ac:dyDescent="0.3">
+      <c r="A10" s="47"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
+      <c r="D10" s="47"/>
+      <c r="E10" s="47"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="47"/>
+      <c r="H10" s="47"/>
+      <c r="I10" s="47"/>
+      <c r="J10" s="47"/>
+    </row>
+    <row r="11" spans="1:10" ht="104" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="87" t="s">
+        <v>515</v>
+      </c>
+      <c r="B11" s="88"/>
+      <c r="C11" s="88"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="88"/>
+      <c r="F11" s="88"/>
+      <c r="G11" s="88"/>
+      <c r="H11" s="88"/>
+      <c r="I11" s="88"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>518</v>
+      </c>
+      <c r="B14" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>0.19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <f>C32</f>
+        <v>71.146490917702906</v>
+      </c>
+      <c r="B18" t="s">
+        <v>534</v>
+      </c>
+      <c r="C18" t="s">
+        <v>522</v>
+      </c>
+      <c r="D18" t="s">
+        <v>523</v>
+      </c>
+      <c r="M18" s="63" t="s">
+        <v>521</v>
+      </c>
+      <c r="N18" s="63"/>
+      <c r="O18" s="63"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C19">
+        <v>25.8</v>
+      </c>
+      <c r="D19">
+        <v>0.5</v>
+      </c>
+      <c r="E19" t="s">
+        <v>524</v>
+      </c>
+      <c r="M19" s="63"/>
+      <c r="N19" s="63"/>
+      <c r="O19" s="63"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C20">
+        <v>59.7</v>
+      </c>
+      <c r="D20">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="E20" t="s">
+        <v>525</v>
+      </c>
+      <c r="M20" s="63"/>
+      <c r="N20" s="63"/>
+      <c r="O20" s="63"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C21">
+        <v>82</v>
+      </c>
+      <c r="D21">
+        <v>0.10199999999999999</v>
+      </c>
+      <c r="E21" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C23" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C24" t="s">
+        <v>528</v>
+      </c>
+      <c r="D24" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" ht="17" x14ac:dyDescent="0.25">
+      <c r="C25" s="48">
+        <v>-7.0092399999999999E-3</v>
+      </c>
+      <c r="D25">
+        <v>0.68868282999999997</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C27" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C28">
+        <f>1/C25</f>
+        <v>-142.66882001472342</v>
+      </c>
+      <c r="D28">
+        <f>D25/C25</f>
+        <v>-98.253566720500359</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C30">
+        <f>D19*C28-D28</f>
+        <v>26.919156713138648</v>
+      </c>
+      <c r="D30" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="C31">
+        <f>D20*C28-D28</f>
+        <v>56.879608916230566</v>
+      </c>
+      <c r="D31" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>531</v>
+      </c>
+      <c r="C32">
+        <f>C28*A17-D28</f>
+        <v>71.146490917702906</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A9:J9"/>
+    <mergeCell ref="A11:I11"/>
+    <mergeCell ref="M18:O20"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10214,10 +10303,10 @@
         <f>intro!B8</f>
         <v>0.68020000000000003</v>
       </c>
-      <c r="M1" s="78" t="s">
+      <c r="M1" s="81" t="s">
         <v>334</v>
       </c>
-      <c r="N1" s="78"/>
+      <c r="N1" s="81"/>
     </row>
     <row r="2" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -10247,11 +10336,11 @@
       <c r="I2">
         <v>36000</v>
       </c>
-      <c r="J2" s="77" t="s">
+      <c r="J2" s="80" t="s">
         <v>327</v>
       </c>
-      <c r="K2" s="77"/>
-      <c r="L2" s="77"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="80"/>
       <c r="M2" s="44" t="s">
         <v>98</v>
       </c>
@@ -10274,16 +10363,16 @@
       <c r="E3">
         <v>947813394500</v>
       </c>
-      <c r="F3" s="77" t="s">
+      <c r="F3" s="80" t="s">
         <v>329</v>
       </c>
       <c r="G3">
         <f>I2/G2</f>
         <v>52925610.114672154</v>
       </c>
-      <c r="J3" s="77"/>
-      <c r="K3" s="77"/>
-      <c r="L3" s="77"/>
+      <c r="J3" s="80"/>
+      <c r="K3" s="80"/>
+      <c r="L3" s="80"/>
       <c r="M3" s="44" t="s">
         <v>333</v>
       </c>
@@ -10307,16 +10396,16 @@
         <f>I4*I5</f>
         <v>45307145.619999997</v>
       </c>
-      <c r="F4" s="77"/>
+      <c r="F4" s="80"/>
       <c r="H4" t="s">
         <v>330</v>
       </c>
       <c r="I4">
         <v>2204.62</v>
       </c>
-      <c r="J4" s="77"/>
-      <c r="K4" s="77"/>
-      <c r="L4" s="77"/>
+      <c r="J4" s="80"/>
+      <c r="K4" s="80"/>
+      <c r="L4" s="80"/>
       <c r="M4" s="44" t="s">
         <v>335</v>
       </c>
@@ -10326,45 +10415,45 @@
       </c>
     </row>
     <row r="5" spans="1:15" ht="53" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F5" s="77"/>
+      <c r="F5" s="80"/>
       <c r="H5" t="s">
         <v>331</v>
       </c>
       <c r="I5">
         <v>20551</v>
       </c>
-      <c r="J5" s="77"/>
-      <c r="K5" s="77"/>
-      <c r="L5" s="77"/>
+      <c r="J5" s="80"/>
+      <c r="K5" s="80"/>
+      <c r="L5" s="80"/>
       <c r="M5" s="44"/>
       <c r="N5" s="44"/>
     </row>
     <row r="6" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="73" t="s">
+      <c r="A6" s="61" t="s">
         <v>142</v>
       </c>
-      <c r="B6" s="73"/>
-      <c r="C6" s="73"/>
-      <c r="D6" s="73"/>
-      <c r="E6" s="73"/>
-      <c r="F6" s="73"/>
-      <c r="G6" s="73"/>
-      <c r="H6" s="73"/>
-      <c r="I6" s="73"/>
-      <c r="J6" s="73"/>
-      <c r="K6" s="73"/>
+      <c r="B6" s="61"/>
+      <c r="C6" s="61"/>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="61"/>
+      <c r="G6" s="61"/>
+      <c r="H6" s="61"/>
+      <c r="I6" s="61"/>
+      <c r="J6" s="61"/>
+      <c r="K6" s="61"/>
       <c r="L6" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="B7" s="67" t="s">
+      <c r="B7" s="64" t="s">
         <v>84</v>
       </c>
-      <c r="C7" s="67"/>
-      <c r="D7" s="67"/>
-      <c r="E7" s="67"/>
-      <c r="F7" s="67"/>
+      <c r="C7" s="64"/>
+      <c r="D7" s="64"/>
+      <c r="E7" s="64"/>
+      <c r="F7" s="64"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="C8" t="s">
@@ -10394,7 +10483,7 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="64" t="s">
+      <c r="A9" s="66" t="s">
         <v>88</v>
       </c>
       <c r="B9" t="s">
@@ -10436,7 +10525,7 @@
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="64"/>
+      <c r="A10" s="66"/>
       <c r="B10" t="s">
         <v>122</v>
       </c>
@@ -10480,7 +10569,7 @@
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="64"/>
+      <c r="A11" s="66"/>
       <c r="B11" t="s">
         <v>123</v>
       </c>
@@ -10520,7 +10609,7 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="64"/>
+      <c r="A12" s="66"/>
       <c r="B12" t="s">
         <v>124</v>
       </c>
@@ -10564,7 +10653,7 @@
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="64"/>
+      <c r="A13" s="66"/>
       <c r="B13" t="s">
         <v>125</v>
       </c>
@@ -10586,7 +10675,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="64" t="s">
+      <c r="A14" s="66" t="s">
         <v>89</v>
       </c>
       <c r="B14" t="s">
@@ -10624,7 +10713,7 @@
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="64"/>
+      <c r="A15" s="66"/>
       <c r="B15" t="s">
         <v>129</v>
       </c>
@@ -10660,7 +10749,7 @@
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="64"/>
+      <c r="A16" s="66"/>
       <c r="B16" t="s">
         <v>126</v>
       </c>
@@ -10696,7 +10785,7 @@
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="64"/>
+      <c r="A17" s="66"/>
       <c r="B17" t="s">
         <v>127</v>
       </c>
@@ -10733,19 +10822,19 @@
     </row>
     <row r="18" spans="1:15" ht="49" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="19" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="73" t="s">
+      <c r="A19" s="61" t="s">
         <v>303</v>
       </c>
-      <c r="B19" s="73"/>
-      <c r="C19" s="73"/>
-      <c r="D19" s="73"/>
-      <c r="E19" s="73"/>
-      <c r="F19" s="73"/>
-      <c r="G19" s="73"/>
-      <c r="H19" s="73"/>
-      <c r="I19" s="73"/>
-      <c r="J19" s="73"/>
-      <c r="K19" s="73"/>
+      <c r="B19" s="61"/>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="61"/>
+      <c r="H19" s="61"/>
+      <c r="I19" s="61"/>
+      <c r="J19" s="61"/>
+      <c r="K19" s="61"/>
     </row>
     <row r="20" spans="1:15" ht="17" x14ac:dyDescent="0.2">
       <c r="A20" s="26" t="s">
@@ -10873,10 +10962,10 @@
       <c r="B34">
         <v>408.31599999999997</v>
       </c>
-      <c r="D34" s="75" t="s">
+      <c r="D34" s="62" t="s">
         <v>309</v>
       </c>
-      <c r="E34" s="75"/>
+      <c r="E34" s="62"/>
       <c r="F34" s="42" t="s">
         <v>109</v>
       </c>
@@ -10917,10 +11006,10 @@
         <f>B34/B35</f>
         <v>1.6789999588798881E-2</v>
       </c>
-      <c r="D36" s="75" t="s">
+      <c r="D36" s="62" t="s">
         <v>313</v>
       </c>
-      <c r="E36" s="75"/>
+      <c r="E36" s="62"/>
       <c r="F36" s="41">
         <f>F35*B36</f>
         <v>3.3579999177597762E-5</v>
@@ -10965,19 +11054,19 @@
       </c>
     </row>
     <row r="40" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="73" t="s">
+      <c r="A40" s="61" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="73"/>
-      <c r="C40" s="73"/>
-      <c r="D40" s="73"/>
-      <c r="E40" s="73"/>
-      <c r="F40" s="73"/>
-      <c r="G40" s="73"/>
-      <c r="H40" s="73"/>
-      <c r="I40" s="73"/>
-      <c r="J40" s="73"/>
-      <c r="K40" s="73"/>
+      <c r="B40" s="61"/>
+      <c r="C40" s="61"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61"/>
+      <c r="F40" s="61"/>
+      <c r="G40" s="61"/>
+      <c r="H40" s="61"/>
+      <c r="I40" s="61"/>
+      <c r="J40" s="61"/>
+      <c r="K40" s="61"/>
     </row>
     <row r="41" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A41" s="26" t="s">
@@ -11478,34 +11567,34 @@
       </c>
     </row>
     <row r="15" spans="1:25" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="73" t="s">
+      <c r="A15" s="61" t="s">
         <v>142</v>
       </c>
-      <c r="B15" s="73"/>
-      <c r="C15" s="73"/>
-      <c r="D15" s="73"/>
-      <c r="E15" s="73"/>
-      <c r="F15" s="73"/>
-      <c r="G15" s="73"/>
-      <c r="H15" s="73"/>
-      <c r="I15" s="73"/>
-      <c r="J15" s="73"/>
-      <c r="K15" s="73"/>
+      <c r="B15" s="61"/>
+      <c r="C15" s="61"/>
+      <c r="D15" s="61"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="61"/>
+      <c r="G15" s="61"/>
+      <c r="H15" s="61"/>
+      <c r="I15" s="61"/>
+      <c r="J15" s="61"/>
+      <c r="K15" s="61"/>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="G16" s="72" t="s">
+      <c r="G16" s="65" t="s">
         <v>100</v>
       </c>
-      <c r="H16" s="72"/>
-      <c r="I16" s="72"/>
-      <c r="J16" s="72"/>
-      <c r="K16" s="72"/>
-      <c r="L16" s="72"/>
-      <c r="N16" s="72" t="s">
+      <c r="H16" s="65"/>
+      <c r="I16" s="65"/>
+      <c r="J16" s="65"/>
+      <c r="K16" s="65"/>
+      <c r="L16" s="65"/>
+      <c r="N16" s="65" t="s">
         <v>101</v>
       </c>
-      <c r="O16" s="72"/>
-      <c r="P16" s="72"/>
+      <c r="O16" s="65"/>
+      <c r="P16" s="65"/>
       <c r="S16" s="23"/>
       <c r="T16" s="23"/>
       <c r="U16" s="23"/>
@@ -12110,19 +12199,19 @@
       </c>
     </row>
     <row r="34" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="73" t="s">
+      <c r="A34" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="B34" s="73"/>
-      <c r="C34" s="73"/>
-      <c r="D34" s="73"/>
-      <c r="E34" s="73"/>
-      <c r="F34" s="73"/>
-      <c r="G34" s="73"/>
-      <c r="H34" s="73"/>
-      <c r="I34" s="73"/>
-      <c r="J34" s="73"/>
-      <c r="K34" s="73"/>
+      <c r="B34" s="61"/>
+      <c r="C34" s="61"/>
+      <c r="D34" s="61"/>
+      <c r="E34" s="61"/>
+      <c r="F34" s="61"/>
+      <c r="G34" s="61"/>
+      <c r="H34" s="61"/>
+      <c r="I34" s="61"/>
+      <c r="J34" s="61"/>
+      <c r="K34" s="61"/>
     </row>
     <row r="35" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="26"/>
@@ -12132,19 +12221,19 @@
     </row>
     <row r="39" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="40" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="73" t="s">
+      <c r="A40" s="61" t="s">
         <v>144</v>
       </c>
-      <c r="B40" s="73"/>
-      <c r="C40" s="73"/>
-      <c r="D40" s="73"/>
-      <c r="E40" s="73"/>
-      <c r="F40" s="73"/>
-      <c r="G40" s="73"/>
-      <c r="H40" s="73"/>
-      <c r="I40" s="73"/>
-      <c r="J40" s="73"/>
-      <c r="K40" s="73"/>
+      <c r="B40" s="61"/>
+      <c r="C40" s="61"/>
+      <c r="D40" s="61"/>
+      <c r="E40" s="61"/>
+      <c r="F40" s="61"/>
+      <c r="G40" s="61"/>
+      <c r="H40" s="61"/>
+      <c r="I40" s="61"/>
+      <c r="J40" s="61"/>
+      <c r="K40" s="61"/>
     </row>
     <row r="42" spans="1:11" ht="17" x14ac:dyDescent="0.2">
       <c r="A42" s="26"/>

</xml_diff>